<commit_message>
[feat] GymLevelData NextLevelId 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/GymLevelData.xlsx
+++ b/JsonConverter/ExcelFiles/GymLevelData.xlsx
@@ -19,12 +19,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="14">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
   <x:si>
-    <x:t>RequiredItem</x:t>
-  </x:si>
-  <x:si>
-    <x:t>gym_level_01</x:t>
+    <x:t>NextLevelId</x:t>
   </x:si>
   <x:si>
     <x:t>int</x:t>
@@ -36,7 +33,16 @@
     <x:t>(name)</x:t>
   </x:si>
   <x:si>
+    <x:t>Level</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
     <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>None</x:t>
   </x:si>
   <x:si>
     <x:t>허름한 체육관</x:t>
@@ -45,22 +51,19 @@
     <x:t>string</x:t>
   </x:si>
   <x:si>
-    <x:t>Name</x:t>
+    <x:t>gym_level_01</x:t>
   </x:si>
   <x:si>
-    <x:t>None</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Level</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GoldCost</x:t>
+    <x:t>RequiredItem</x:t>
   </x:si>
   <x:si>
     <x:t>Description</x:t>
   </x:si>
   <x:si>
     <x:t>시작 체육관이다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GoldCost</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -814,7 +817,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:F35"/>
+  <x:dimension ref="A1:G35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="16.28515625" style="1" customWidth="1"/>
@@ -830,58 +833,64 @@
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>5</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" spans="1:6" ht="13.199999999999999">
+    <x:row r="2" spans="1:7" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:7" s="6" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="2" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:6" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="2" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>10</x:v>
-      </x:c>
       <x:c r="C3" s="2" t="s">
-        <x:v>8</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D3" s="2" t="s">
         <x:v>12</x:v>
       </x:c>
       <x:c r="E3" s="6" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="s">
         <x:v>11</x:v>
       </x:c>
-      <x:c r="F3" s="6" t="s">
+      <x:c r="G3" s="6" t="s">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>1</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B4" s="3">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>6</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
         <x:v>13</x:v>
@@ -890,7 +899,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="F4" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:3" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
[feat] GymLevelData Type과 휴식 공간 추가
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/GymLevelData.xlsx
+++ b/JsonConverter/ExcelFiles/GymLevelData.xlsx
@@ -19,51 +19,90 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
+  <x:si>
+    <x:t>선수 육성을 시작한 체육관이다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>낡고 보잘것 없는 휴식 공간이다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gym</x:t>
+  </x:si>
+  <x:si>
+    <x:t>1W</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rest</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Type</x:t>
+  </x:si>
+  <x:si>
+    <x:t>허름한 체육관</x:t>
+  </x:si>
+  <x:si>
+    <x:t>낡은 체육관</x:t>
+  </x:si>
+  <x:si>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
+  </x:si>
+  <x:si>
+    <x:t>None</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Level</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rest_level_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rest_level_02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gym_level_01</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gym_level_02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiredItem</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GoldCost</x:t>
+  </x:si>
   <x:si>
     <x:t>NextLevelId</x:t>
   </x:si>
   <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Level</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>None</x:t>
-  </x:si>
-  <x:si>
-    <x:t>허름한 체육관</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>gym_level_01</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RequiredItem</x:t>
-  </x:si>
-  <x:si>
     <x:t>Description</x:t>
   </x:si>
   <x:si>
     <x:t>시작 체육관이다.</x:t>
   </x:si>
   <x:si>
-    <x:t>GoldCost</x:t>
+    <x:t>낡은 휴식 공간</x:t>
+  </x:si>
+  <x:si>
+    <x:t>좁은 휴식 공간</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개선되었지만 여전히 좁고 불편한 휴식 공간이다.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -817,105 +856,183 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetPr codeName="Sheet1"/>
-  <x:dimension ref="A1:G35"/>
+  <x:dimension ref="A1:H35"/>
   <x:sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15" customHeight="1"/>
   <x:cols>
     <x:col min="1" max="1" width="16.28515625" style="1" customWidth="1"/>
-    <x:col min="2" max="2" width="19.54296875" style="1" customWidth="1"/>
-    <x:col min="3" max="3" width="41" style="1" customWidth="1"/>
+    <x:col min="2" max="2" width="17.14453125" style="1" customWidth="1"/>
+    <x:col min="3" max="3" width="14" style="1" customWidth="1"/>
     <x:col min="4" max="4" width="26.4296875" style="1" customWidth="1"/>
-    <x:col min="5" max="5" width="30.54296875" style="1" customWidth="1"/>
+    <x:col min="5" max="5" width="41.71484375" style="1" customWidth="1"/>
     <x:col min="6" max="6" width="26.54296875" style="1" customWidth="1"/>
     <x:col min="7" max="7" width="20" style="1" customWidth="1"/>
-    <x:col min="8" max="12" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
+    <x:col min="8" max="8" width="21.28515625" style="1" customWidth="1"/>
+    <x:col min="9" max="9" width="16.28515625" style="1" customWidth="1"/>
+    <x:col min="10" max="10" width="17.5703125" style="1" customWidth="1"/>
+    <x:col min="11" max="12" width="12.54296875" style="1" bestFit="1" customWidth="1"/>
     <x:col min="13" max="16384" width="12.54296875" style="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:1" ht="15.75" customHeight="1">
       <x:c r="A1" s="1" t="s">
+        <x:v>11</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:8" ht="13.199999999999999">
+      <x:c r="A2" s="1" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="C2" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F2" s="1" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="G2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="H2" s="1" t="s">
+        <x:v>10</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:8" s="6" customFormat="1" ht="15.75" customHeight="1">
+      <x:c r="A3" s="2" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="2" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="C3" s="2" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D3" s="2" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="E3" s="2" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="F3" s="6" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="G3" s="6" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="H3" s="6" t="s">
+        <x:v>22</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:8" ht="15.75" customHeight="1">
+      <x:c r="A4" s="3" t="s">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C4" s="3">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D4" s="3" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E4" s="3" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="F4" s="1">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G4" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H4" s="1" t="s">
+        <x:v>19</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:8" ht="15.75" customHeight="1">
+      <x:c r="A5" s="3" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B5" s="3" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C5" s="3">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D5" s="1" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E5" s="1" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="1">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="G5" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="H5" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:8" ht="15.75" customHeight="1">
+      <x:c r="A6" s="3" t="s">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B6" s="4" t="s">
         <x:v>6</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:7" ht="13.199999999999999">
-      <x:c r="A2" s="1" t="s">
+      <x:c r="C6" s="4">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="D6" s="1" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="E6" s="1" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F6" s="1">
+        <x:v>500</x:v>
+      </x:c>
+      <x:c r="G6" s="1" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B2" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C2" s="1" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="D2" s="1" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="E2" s="1" t="s">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F2" s="1" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="G2" s="1" t="s">
-        <x:v>9</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:7" s="6" customFormat="1" ht="15.75" customHeight="1">
-      <x:c r="A3" s="2" t="s">
+      <x:c r="H6" s="1" t="s">
+        <x:v>17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:8" ht="15.75" customHeight="1">
+      <x:c r="A7" s="4" t="s">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B7" s="4" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C7" s="4">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B3" s="2" t="s">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C3" s="2" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D3" s="2" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="E3" s="6" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="F3" s="6" t="s">
-        <x:v>11</x:v>
-      </x:c>
-      <x:c r="G3" s="6" t="s">
-        <x:v>0</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:6" ht="15.75" customHeight="1">
-      <x:c r="A4" s="3" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="B4" s="3">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C4" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="D4" s="3" t="s">
+      <x:c r="D7" s="1" t="s">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="E7" s="1" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F7" s="1">
+        <x:v>1500</x:v>
+      </x:c>
+      <x:c r="G7" s="1" t="s">
         <x:v>13</x:v>
       </x:c>
-      <x:c r="E4" s="1">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F4" s="1" t="s">
-        <x:v>7</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A5" s="3"/>
-      <x:c r="B5" s="3"/>
-      <x:c r="C5" s="3"/>
-    </x:row>
-    <x:row r="6" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A6" s="3"/>
-      <x:c r="B6" s="4"/>
-      <x:c r="C6" s="4"/>
-    </x:row>
-    <x:row r="7" spans="1:3" ht="15.75" customHeight="1">
-      <x:c r="A7" s="4"/>
-      <x:c r="B7" s="4"/>
-      <x:c r="C7" s="4"/>
+      <x:c r="H7" s="1" t="s">
+        <x:v>13</x:v>
+      </x:c>
     </x:row>
     <x:row r="8" spans="1:3" ht="15.75" customHeight="1">
       <x:c r="A8" s="4"/>

</xml_diff>

<commit_message>
[feat] 해금 조건을 RequiredUnlockIds로 연결
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/GymLevelData.xlsx
+++ b/JsonConverter/ExcelFiles/GymLevelData.xlsx
@@ -19,90 +19,93 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
+<x:sst xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="29">
+  <x:si>
+    <x:t>cond_win_1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gym</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Id</x:t>
+  </x:si>
+  <x:si>
+    <x:t>int</x:t>
+  </x:si>
+  <x:si>
+    <x:t>RequiredUnlockIds</x:t>
+  </x:si>
+  <x:si>
+    <x:t>낡고 보잘것 없는 휴식 공간이다.</x:t>
+  </x:si>
   <x:si>
     <x:t>선수 육성을 시작한 체육관이다.</x:t>
   </x:si>
   <x:si>
-    <x:t>낡고 보잘것 없는 휴식 공간이다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>gym</x:t>
-  </x:si>
-  <x:si>
-    <x:t>1W</x:t>
-  </x:si>
-  <x:si>
-    <x:t>int</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Id</x:t>
+    <x:t>string</x:t>
+  </x:si>
+  <x:si>
+    <x:t>낡은 체육관</x:t>
+  </x:si>
+  <x:si>
+    <x:t>None</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Level</x:t>
+  </x:si>
+  <x:si>
+    <x:t>고유 ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Name</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Type</x:t>
+  </x:si>
+  <x:si>
+    <x:t>(name)</x:t>
   </x:si>
   <x:si>
     <x:t>rest</x:t>
   </x:si>
   <x:si>
-    <x:t>Type</x:t>
-  </x:si>
-  <x:si>
     <x:t>허름한 체육관</x:t>
   </x:si>
   <x:si>
-    <x:t>낡은 체육관</x:t>
-  </x:si>
-  <x:si>
-    <x:t>string</x:t>
-  </x:si>
-  <x:si>
-    <x:t>고유 ID</x:t>
-  </x:si>
-  <x:si>
-    <x:t>(name)</x:t>
-  </x:si>
-  <x:si>
-    <x:t>None</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Level</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Name</x:t>
+    <x:t>NextLevelId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>GoldCost</x:t>
+  </x:si>
+  <x:si>
+    <x:t>시작 체육관이다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Description</x:t>
+  </x:si>
+  <x:si>
+    <x:t>좁은 휴식 공간</x:t>
+  </x:si>
+  <x:si>
+    <x:t>낡은 휴식 공간</x:t>
+  </x:si>
+  <x:si>
+    <x:t>개선되었지만 여전히 좁고 불편한 휴식 공간이다.</x:t>
+  </x:si>
+  <x:si>
+    <x:t>cond_streak_3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>rest_level_02</x:t>
+  </x:si>
+  <x:si>
+    <x:t>gym_level_01</x:t>
   </x:si>
   <x:si>
     <x:t>rest_level_01</x:t>
   </x:si>
   <x:si>
-    <x:t>rest_level_02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>gym_level_01</x:t>
-  </x:si>
-  <x:si>
     <x:t>gym_level_02</x:t>
-  </x:si>
-  <x:si>
-    <x:t>RequiredItem</x:t>
-  </x:si>
-  <x:si>
-    <x:t>GoldCost</x:t>
-  </x:si>
-  <x:si>
-    <x:t>NextLevelId</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Description</x:t>
-  </x:si>
-  <x:si>
-    <x:t>시작 체육관이다.</x:t>
-  </x:si>
-  <x:si>
-    <x:t>낡은 휴식 공간</x:t>
-  </x:si>
-  <x:si>
-    <x:t>좁은 휴식 공간</x:t>
-  </x:si>
-  <x:si>
-    <x:t>개선되었지만 여전히 좁고 불편한 휴식 공간이다.</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -865,7 +868,7 @@
     <x:col min="4" max="4" width="26.4296875" style="1" customWidth="1"/>
     <x:col min="5" max="5" width="41.71484375" style="1" customWidth="1"/>
     <x:col min="6" max="6" width="26.54296875" style="1" customWidth="1"/>
-    <x:col min="7" max="7" width="20" style="1" customWidth="1"/>
+    <x:col min="7" max="7" width="42.14453125" style="1" customWidth="1"/>
     <x:col min="8" max="8" width="21.28515625" style="1" customWidth="1"/>
     <x:col min="9" max="9" width="16.28515625" style="1" customWidth="1"/>
     <x:col min="10" max="10" width="17.5703125" style="1" customWidth="1"/>
@@ -880,158 +883,158 @@
     </x:row>
     <x:row r="2" spans="1:8" ht="13.199999999999999">
       <x:c r="A2" s="1" t="s">
-        <x:v>12</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C2" s="1" t="s">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="F2" s="1" t="s">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="G2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="H2" s="1" t="s">
-        <x:v>10</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8" s="6" customFormat="1" ht="15.75" customHeight="1">
       <x:c r="A3" s="2" t="s">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B3" s="2" t="s">
-        <x:v>7</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C3" s="2" t="s">
-        <x:v>14</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="D3" s="2" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="E3" s="2" t="s">
-        <x:v>23</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F3" s="6" t="s">
-        <x:v>21</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="G3" s="6" t="s">
-        <x:v>20</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="H3" s="6" t="s">
-        <x:v>22</x:v>
+        <x:v>17</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A4" s="3" t="s">
-        <x:v>18</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C4" s="3">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>8</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="E4" s="3" t="s">
-        <x:v>24</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="F4" s="1">
         <x:v>0</x:v>
       </x:c>
       <x:c r="G4" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H4" s="1" t="s">
-        <x:v>19</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
-        <x:v>19</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="C5" s="3">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D5" s="1" t="s">
-        <x:v>9</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E5" s="1" t="s">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="F5" s="1">
         <x:v>1000</x:v>
       </x:c>
       <x:c r="G5" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="H5" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A6" s="3" t="s">
-        <x:v>16</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="B6" s="4" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C6" s="4">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D6" s="1" t="s">
-        <x:v>25</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="E6" s="1" t="s">
-        <x:v>1</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="F6" s="1">
         <x:v>500</x:v>
       </x:c>
       <x:c r="G6" s="1" t="s">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H6" s="1" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:8" ht="15.75" customHeight="1">
       <x:c r="A7" s="4" t="s">
-        <x:v>17</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="B7" s="4" t="s">
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C7" s="4">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D7" s="1" t="s">
-        <x:v>26</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E7" s="1" t="s">
-        <x:v>27</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="F7" s="1">
         <x:v>1500</x:v>
       </x:c>
       <x:c r="G7" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="H7" s="1" t="s">
-        <x:v>13</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:3" ht="15.75" customHeight="1">

</xml_diff>